<commit_message>
docs(xlsx): convert facturación column to PV/mes (1 PV = $2 USD)
- Column "Facturación estructura/mes" → "PV/mes"
- Values halved (1 PV = $2): $2,000 → 1,000 PV ... $2,500,000 → 1,250,000 PV
- Number format changed from "$"#,##0 to #,##0" PV" (no $ symbol)
- Added "PV (Punto de Volumen)" definition with $2 equivalence
- Adjusted PV/mes column width to 16

PV mínimo column kept in USD for now per user instruction (will be
converted in next iteration along with bonus percentages).

https://claude.ai/code/session_01SAeJFAFBsbYi7asgp8AEPk
</commit_message>
<xml_diff>
--- a/docs/requisitos-calificacion.xlsx
+++ b/docs/requisitos-calificacion.xlsx
@@ -16,8 +16,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
+  <numFmts count="2">
+    <numFmt numFmtId="164" formatCode="#,##0&quot; PV&quot;"/>
+    <numFmt numFmtId="165" formatCode="&quot;$&quot;#,##0"/>
   </numFmts>
   <fonts count="12">
     <font>
@@ -152,7 +153,7 @@
     <xf numFmtId="164" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -167,7 +168,7 @@
     <xf numFmtId="164" fontId="6" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -182,7 +183,7 @@
     <xf numFmtId="164" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -563,12 +564,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G30"/>
+  <dimension ref="A1:G32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
     <col width="22" customWidth="1" min="2" max="2"/>
-    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
     <col width="18" customWidth="1" min="6" max="6"/>
@@ -603,7 +604,7 @@
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>Facturación estructura/mes</t>
+          <t>PV/mes</t>
         </is>
       </c>
       <c r="D4" s="3" t="inlineStr">
@@ -637,7 +638,7 @@
         </is>
       </c>
       <c r="C5" s="6" t="n">
-        <v>2000</v>
+        <v>1000</v>
       </c>
       <c r="D5" s="7" t="n">
         <v>200</v>
@@ -666,7 +667,7 @@
         </is>
       </c>
       <c r="C6" s="6" t="n">
-        <v>4000</v>
+        <v>2000</v>
       </c>
       <c r="D6" s="7" t="n">
         <v>200</v>
@@ -695,7 +696,7 @@
         </is>
       </c>
       <c r="C7" s="6" t="n">
-        <v>8000</v>
+        <v>4000</v>
       </c>
       <c r="D7" s="7" t="n">
         <v>300</v>
@@ -724,7 +725,7 @@
         </is>
       </c>
       <c r="C8" s="6" t="n">
-        <v>15000</v>
+        <v>7500</v>
       </c>
       <c r="D8" s="7" t="n">
         <v>300</v>
@@ -753,7 +754,7 @@
         </is>
       </c>
       <c r="C9" s="6" t="n">
-        <v>25000</v>
+        <v>12500</v>
       </c>
       <c r="D9" s="7" t="n">
         <v>400</v>
@@ -782,7 +783,7 @@
         </is>
       </c>
       <c r="C10" s="6" t="n">
-        <v>40000</v>
+        <v>20000</v>
       </c>
       <c r="D10" s="7" t="n">
         <v>500</v>
@@ -811,7 +812,7 @@
         </is>
       </c>
       <c r="C11" s="6" t="n">
-        <v>80000</v>
+        <v>40000</v>
       </c>
       <c r="D11" s="7" t="n">
         <v>500</v>
@@ -840,7 +841,7 @@
         </is>
       </c>
       <c r="C12" s="6" t="n">
-        <v>150000</v>
+        <v>75000</v>
       </c>
       <c r="D12" s="7" t="n">
         <v>500</v>
@@ -869,7 +870,7 @@
         </is>
       </c>
       <c r="C13" s="11" t="n">
-        <v>250000</v>
+        <v>125000</v>
       </c>
       <c r="D13" s="12" t="n">
         <v>1000</v>
@@ -898,7 +899,7 @@
         </is>
       </c>
       <c r="C14" s="11" t="n">
-        <v>500000</v>
+        <v>250000</v>
       </c>
       <c r="D14" s="12" t="n">
         <v>1000</v>
@@ -927,7 +928,7 @@
         </is>
       </c>
       <c r="C15" s="11" t="n">
-        <v>1000000</v>
+        <v>500000</v>
       </c>
       <c r="D15" s="12" t="n">
         <v>1000</v>
@@ -956,7 +957,7 @@
         </is>
       </c>
       <c r="C16" s="16" t="n">
-        <v>2500000</v>
+        <v>1250000</v>
       </c>
       <c r="D16" s="17" t="n">
         <v>1000</v>
@@ -985,111 +986,137 @@
     <row r="20" ht="22" customHeight="1">
       <c r="A20" s="20" t="inlineStr">
         <is>
-          <t>PV (Volumen Personal)</t>
+          <t>PV (Punto de Volumen)</t>
         </is>
       </c>
       <c r="B20" s="21" t="inlineStr">
         <is>
-          <t>Ventas que TÚ cierras directamente con clientes/socios.</t>
+          <t>Unidad de medida del plan. Equivalencia oficial: 1 PV = $2 USD.</t>
         </is>
       </c>
     </row>
     <row r="21" ht="22" customHeight="1">
       <c r="A21" s="20" t="inlineStr">
         <is>
-          <t>Patrocinados activos</t>
+          <t>PV/mes</t>
         </is>
       </c>
       <c r="B21" s="21" t="inlineStr">
         <is>
-          <t>Socios que TÚ trajiste personalmente y que cumplen su PV mínimo ese mes.</t>
+          <t>Volumen total facturado por toda tu estructura en el mes (en puntos).</t>
         </is>
       </c>
     </row>
     <row r="22" ht="22" customHeight="1">
       <c r="A22" s="20" t="inlineStr">
         <is>
-          <t>Piernas calificadas</t>
+          <t>PV mínimo</t>
         </is>
       </c>
       <c r="B22" s="21" t="inlineStr">
         <is>
-          <t>Ramas independientes (downlines de patrocinados directos distintos) donde alguien dentro alcanza el rango indicado entre paréntesis.</t>
+          <t>Volumen Personal mínimo que TÚ debes producir directamente cada mes (pendiente: convertir a puntos en próxima iteración).</t>
         </is>
       </c>
     </row>
     <row r="23" ht="22" customHeight="1">
       <c r="A23" s="20" t="inlineStr">
         <is>
-          <t>Cobro estimado</t>
+          <t>Patrocinados activos</t>
         </is>
       </c>
       <c r="B23" s="21" t="inlineStr">
         <is>
-          <t>Ingreso aproximado mensual proyectado por la combinación FSB + Uninivel + Pool.</t>
+          <t>Socios que TÚ trajiste personalmente y que cumplen su PV mínimo ese mes.</t>
         </is>
       </c>
     </row>
     <row r="24" ht="22" customHeight="1">
       <c r="A24" s="20" t="inlineStr">
         <is>
+          <t>Piernas calificadas</t>
+        </is>
+      </c>
+      <c r="B24" s="21" t="inlineStr">
+        <is>
+          <t>Ramas independientes (downlines de patrocinados directos distintos) donde alguien dentro alcanza el rango indicado entre paréntesis.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="22" customHeight="1">
+      <c r="A25" s="20" t="inlineStr">
+        <is>
+          <t>Cobro estimado</t>
+        </is>
+      </c>
+      <c r="B25" s="21" t="inlineStr">
+        <is>
+          <t>Ingreso aproximado mensual proyectado por la combinación FSB + Uninivel + Pool.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="22" customHeight="1">
+      <c r="A26" s="20" t="inlineStr">
+        <is>
           <t>Regla 50/50 (sugerida)</t>
         </is>
       </c>
-      <c r="B24" s="21" t="inlineStr">
+      <c r="B26" s="21" t="inlineStr">
         <is>
           <t>Ninguna pierna puede aportar más del 50% del volumen requerido para el rango.</t>
         </is>
       </c>
     </row>
-    <row r="26">
-      <c r="A26" s="19" t="inlineStr">
+    <row r="28">
+      <c r="A28" s="19" t="inlineStr">
         <is>
           <t>PENDIENTES DE CONFIRMAR</t>
-        </is>
-      </c>
-    </row>
-    <row r="27" ht="20" customHeight="1">
-      <c r="A27" s="22" t="inlineStr">
-        <is>
-          <t>☐  PV mínimos por rango (¿OK los valores propuestos?)</t>
-        </is>
-      </c>
-    </row>
-    <row r="28" ht="20" customHeight="1">
-      <c r="A28" s="22" t="inlineStr">
-        <is>
-          <t>☐  Número de patrocinados activos por rango</t>
         </is>
       </c>
     </row>
     <row r="29" ht="20" customHeight="1">
       <c r="A29" s="22" t="inlineStr">
         <is>
-          <t>☐  Piernas calificadas y su rango exigido</t>
+          <t>☐  PV mínimos por rango (¿OK los valores propuestos?)</t>
         </is>
       </c>
     </row>
     <row r="30" ht="20" customHeight="1">
       <c r="A30" s="22" t="inlineStr">
         <is>
+          <t>☐  Número de patrocinados activos por rango</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="20" customHeight="1">
+      <c r="A31" s="22" t="inlineStr">
+        <is>
+          <t>☐  Piernas calificadas y su rango exigido</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="20" customHeight="1">
+      <c r="A32" s="22" t="inlineStr">
+        <is>
           <t>☐  Activar/no activar regla 50/50</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="11">
+  <mergeCells count="13">
     <mergeCell ref="B24:G24"/>
+    <mergeCell ref="A32:G32"/>
     <mergeCell ref="B20:G20"/>
     <mergeCell ref="A1:G1"/>
     <mergeCell ref="B22:G22"/>
-    <mergeCell ref="A27:G27"/>
+    <mergeCell ref="A31:G31"/>
     <mergeCell ref="B23:G23"/>
     <mergeCell ref="A30:G30"/>
     <mergeCell ref="A2:G2"/>
+    <mergeCell ref="B26:G26"/>
     <mergeCell ref="A29:G29"/>
     <mergeCell ref="B21:G21"/>
-    <mergeCell ref="A28:G28"/>
+    <mergeCell ref="B25:G25"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter>

</xml_diff>

<commit_message>
docs(xlsx): add Bono Gift column + formula-based Cobro estimado
- New "Bono Gift" column (G) — editable, default $0, blue highlight
  to indicate input cell
- "Cobro estimado" (H) is now a FORMULA cell:
  Min = 22% × PV/mes (current rank) + Bono Gift
  Max = 22% × PV/mes (next rank)    + Bono Gift
  Leyenda shows only "$X+" with no upper bound
- When user edits Bono Gift, Cobro auto-recalculates (both min & max)
- Updated definitions section with Bono Gift and Cobro formula docs
- Adjusted column widths and merged ranges for the new 8th column

https://claude.ai/code/session_01SAeJFAFBsbYi7asgp8AEPk
</commit_message>
<xml_diff>
--- a/docs/requisitos-calificacion.xlsx
+++ b/docs/requisitos-calificacion.xlsx
@@ -20,7 +20,7 @@
     <numFmt numFmtId="164" formatCode="#,##0&quot; PV&quot;"/>
     <numFmt numFmtId="165" formatCode="&quot;$&quot;#,##0"/>
   </numFmts>
-  <fonts count="12">
+  <fonts count="13">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -64,6 +64,12 @@
     <font>
       <name val="Calibri"/>
       <b val="1"/>
+      <color rgb="000066CC"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
       <color rgb="002E7D32"/>
       <sz val="11"/>
     </font>
@@ -84,7 +90,7 @@
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="8">
     <fill>
       <patternFill/>
     </fill>
@@ -98,12 +104,27 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="00EAF4FF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="00FFF8E8"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="00FFF3D6"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="00FCE4A6"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FCDD8E"/>
       </patternFill>
     </fill>
   </fills>
@@ -133,7 +154,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="26">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -156,22 +177,10 @@
     <xf numFmtId="165" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="7" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -186,17 +195,38 @@
     <xf numFmtId="165" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="7" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="4" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="7" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" indent="1"/>
     </xf>
   </cellXfs>
@@ -564,7 +594,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G32"/>
+  <dimension ref="A1:H33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -573,7 +603,8 @@
     <col width="12" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
     <col width="18" customWidth="1" min="6" max="6"/>
-    <col width="22" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="22" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
@@ -624,6 +655,11 @@
       </c>
       <c r="G4" s="3" t="inlineStr">
         <is>
+          <t>Bono Gift</t>
+        </is>
+      </c>
+      <c r="H4" s="3" t="inlineStr">
+        <is>
           <t>Cobro estimado</t>
         </is>
       </c>
@@ -651,10 +687,12 @@
           <t>—</t>
         </is>
       </c>
-      <c r="G5" s="8" t="inlineStr">
-        <is>
-          <t>$220 – $439</t>
-        </is>
+      <c r="G5" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="H5" s="9">
+        <f>TEXT(INT(0.22*C5)+G5,"$#,##0")&amp;" – "&amp;TEXT(INT(0.22*C6)+G5,"$#,##0")</f>
+        <v/>
       </c>
     </row>
     <row r="6" ht="26" customHeight="1">
@@ -680,10 +718,12 @@
           <t>—</t>
         </is>
       </c>
-      <c r="G6" s="8" t="inlineStr">
-        <is>
-          <t>$440 – $879</t>
-        </is>
+      <c r="G6" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="H6" s="9">
+        <f>TEXT(INT(0.22*C6)+G6,"$#,##0")&amp;" – "&amp;TEXT(INT(0.22*C7)+G6,"$#,##0")</f>
+        <v/>
       </c>
     </row>
     <row r="7" ht="26" customHeight="1">
@@ -709,10 +749,12 @@
           <t>1 (Ejecutivo+)</t>
         </is>
       </c>
-      <c r="G7" s="8" t="inlineStr">
-        <is>
-          <t>$880 – $1,649</t>
-        </is>
+      <c r="G7" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="H7" s="9">
+        <f>TEXT(INT(0.22*C7)+G7,"$#,##0")&amp;" – "&amp;TEXT(INT(0.22*C8)+G7,"$#,##0")</f>
+        <v/>
       </c>
     </row>
     <row r="8" ht="26" customHeight="1">
@@ -738,10 +780,12 @@
           <t>2 (Ejecutivo+)</t>
         </is>
       </c>
-      <c r="G8" s="8" t="inlineStr">
-        <is>
-          <t>$1,650 – $2,749</t>
-        </is>
+      <c r="G8" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="H8" s="9">
+        <f>TEXT(INT(0.22*C8)+G8,"$#,##0")&amp;" – "&amp;TEXT(INT(0.22*C9)+G8,"$#,##0")</f>
+        <v/>
       </c>
     </row>
     <row r="9" ht="26" customHeight="1">
@@ -767,10 +811,12 @@
           <t>2 (D1500+)</t>
         </is>
       </c>
-      <c r="G9" s="8" t="inlineStr">
-        <is>
-          <t>$2,750 – $4,399</t>
-        </is>
+      <c r="G9" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="H9" s="9">
+        <f>TEXT(INT(0.22*C9)+G9,"$#,##0")&amp;" – "&amp;TEXT(INT(0.22*C10)+G9,"$#,##0")</f>
+        <v/>
       </c>
     </row>
     <row r="10" ht="26" customHeight="1">
@@ -796,10 +842,12 @@
           <t>3 (D1500+)</t>
         </is>
       </c>
-      <c r="G10" s="8" t="inlineStr">
-        <is>
-          <t>$4,400 – $8,799</t>
-        </is>
+      <c r="G10" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="H10" s="9">
+        <f>TEXT(INT(0.22*C10)+G10,"$#,##0")&amp;" – "&amp;TEXT(INT(0.22*C11)+G10,"$#,##0")</f>
+        <v/>
       </c>
     </row>
     <row r="11" ht="26" customHeight="1">
@@ -825,10 +873,12 @@
           <t>3 (D2500+)</t>
         </is>
       </c>
-      <c r="G11" s="8" t="inlineStr">
-        <is>
-          <t>$8,800 – $16,499</t>
-        </is>
+      <c r="G11" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="H11" s="9">
+        <f>TEXT(INT(0.22*C11)+G11,"$#,##0")&amp;" – "&amp;TEXT(INT(0.22*C12)+G11,"$#,##0")</f>
+        <v/>
       </c>
     </row>
     <row r="12" ht="26" customHeight="1">
@@ -854,269 +904,292 @@
           <t>3 (D4K+)</t>
         </is>
       </c>
-      <c r="G12" s="8" t="inlineStr">
-        <is>
-          <t>$16,500 – $27,499</t>
-        </is>
+      <c r="G12" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="H12" s="9">
+        <f>TEXT(INT(0.22*C12)+G12,"$#,##0")&amp;" – "&amp;TEXT(INT(0.22*C13)+G12,"$#,##0")</f>
+        <v/>
       </c>
     </row>
     <row r="13" ht="26" customHeight="1">
-      <c r="A13" s="9" t="n">
+      <c r="A13" s="10" t="n">
         <v>9</v>
       </c>
-      <c r="B13" s="10" t="inlineStr">
+      <c r="B13" s="11" t="inlineStr">
         <is>
           <t>Embajador Elite 30K</t>
         </is>
       </c>
-      <c r="C13" s="11" t="n">
+      <c r="C13" s="12" t="n">
         <v>125000</v>
       </c>
-      <c r="D13" s="12" t="n">
+      <c r="D13" s="13" t="n">
         <v>1000</v>
       </c>
-      <c r="E13" s="9" t="n">
+      <c r="E13" s="10" t="n">
         <v>6</v>
       </c>
-      <c r="F13" s="9" t="inlineStr">
+      <c r="F13" s="10" t="inlineStr">
         <is>
           <t>3 (P7K+)</t>
         </is>
       </c>
-      <c r="G13" s="13" t="inlineStr">
-        <is>
-          <t>$27,500 – $54,999</t>
-        </is>
+      <c r="G13" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="H13" s="15">
+        <f>TEXT(INT(0.22*C13)+G13,"$#,##0")&amp;" – "&amp;TEXT(INT(0.22*C14)+G13,"$#,##0")</f>
+        <v/>
       </c>
     </row>
     <row r="14" ht="26" customHeight="1">
-      <c r="A14" s="9" t="n">
+      <c r="A14" s="10" t="n">
         <v>10</v>
       </c>
-      <c r="B14" s="10" t="inlineStr">
+      <c r="B14" s="11" t="inlineStr">
         <is>
           <t>Embajador Corona 60K</t>
         </is>
       </c>
-      <c r="C14" s="11" t="n">
+      <c r="C14" s="12" t="n">
         <v>250000</v>
       </c>
-      <c r="D14" s="12" t="n">
+      <c r="D14" s="13" t="n">
         <v>1000</v>
       </c>
-      <c r="E14" s="9" t="n">
+      <c r="E14" s="10" t="n">
         <v>6</v>
       </c>
-      <c r="F14" s="9" t="inlineStr">
+      <c r="F14" s="10" t="inlineStr">
         <is>
           <t>3 (P15K+)</t>
         </is>
       </c>
-      <c r="G14" s="13" t="inlineStr">
-        <is>
-          <t>$55,000 – $109,999</t>
-        </is>
+      <c r="G14" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="H14" s="15">
+        <f>TEXT(INT(0.22*C14)+G14,"$#,##0")&amp;" – "&amp;TEXT(INT(0.22*C15)+G14,"$#,##0")</f>
+        <v/>
       </c>
     </row>
     <row r="15" ht="26" customHeight="1">
-      <c r="A15" s="9" t="n">
+      <c r="A15" s="10" t="n">
         <v>11</v>
       </c>
-      <c r="B15" s="10" t="inlineStr">
+      <c r="B15" s="11" t="inlineStr">
         <is>
           <t>Icon 120K</t>
         </is>
       </c>
-      <c r="C15" s="11" t="n">
+      <c r="C15" s="12" t="n">
         <v>500000</v>
       </c>
-      <c r="D15" s="12" t="n">
+      <c r="D15" s="13" t="n">
         <v>1000</v>
       </c>
-      <c r="E15" s="9" t="n">
+      <c r="E15" s="10" t="n">
         <v>6</v>
       </c>
-      <c r="F15" s="9" t="inlineStr">
+      <c r="F15" s="10" t="inlineStr">
         <is>
           <t>3 (P25K+)</t>
         </is>
       </c>
-      <c r="G15" s="13" t="inlineStr">
-        <is>
-          <t>$110,000 – $274,999</t>
-        </is>
+      <c r="G15" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="H15" s="15">
+        <f>TEXT(INT(0.22*C15)+G15,"$#,##0")&amp;" – "&amp;TEXT(INT(0.22*C16)+G15,"$#,##0")</f>
+        <v/>
       </c>
     </row>
     <row r="16" ht="26" customHeight="1">
-      <c r="A16" s="14" t="n">
+      <c r="A16" s="16" t="n">
         <v>12</v>
       </c>
-      <c r="B16" s="15" t="inlineStr">
+      <c r="B16" s="17" t="inlineStr">
         <is>
           <t>Leyenda 300K</t>
         </is>
       </c>
-      <c r="C16" s="16" t="n">
+      <c r="C16" s="18" t="n">
         <v>1250000</v>
       </c>
-      <c r="D16" s="17" t="n">
+      <c r="D16" s="19" t="n">
         <v>1000</v>
       </c>
-      <c r="E16" s="14" t="n">
+      <c r="E16" s="16" t="n">
         <v>6</v>
       </c>
-      <c r="F16" s="14" t="inlineStr">
+      <c r="F16" s="16" t="inlineStr">
         <is>
           <t>3 (Embajador+)</t>
         </is>
       </c>
-      <c r="G16" s="18" t="inlineStr">
-        <is>
-          <t>$275,000+</t>
-        </is>
+      <c r="G16" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="H16" s="21">
+        <f>TEXT(INT(0.22*C16)+G16,"$#,##0")&amp;"+"</f>
+        <v/>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="19" t="inlineStr">
+      <c r="A19" s="22" t="inlineStr">
         <is>
           <t>DEFINICIONES</t>
         </is>
       </c>
     </row>
     <row r="20" ht="22" customHeight="1">
-      <c r="A20" s="20" t="inlineStr">
+      <c r="A20" s="23" t="inlineStr">
         <is>
           <t>PV (Punto de Volumen)</t>
         </is>
       </c>
-      <c r="B20" s="21" t="inlineStr">
+      <c r="B20" s="24" t="inlineStr">
         <is>
           <t>Unidad de medida del plan. Equivalencia oficial: 1 PV = $2 USD.</t>
         </is>
       </c>
     </row>
     <row r="21" ht="22" customHeight="1">
-      <c r="A21" s="20" t="inlineStr">
+      <c r="A21" s="23" t="inlineStr">
         <is>
           <t>PV/mes</t>
         </is>
       </c>
-      <c r="B21" s="21" t="inlineStr">
+      <c r="B21" s="24" t="inlineStr">
         <is>
           <t>Volumen total facturado por toda tu estructura en el mes (en puntos).</t>
         </is>
       </c>
     </row>
     <row r="22" ht="22" customHeight="1">
-      <c r="A22" s="20" t="inlineStr">
+      <c r="A22" s="23" t="inlineStr">
         <is>
           <t>PV mínimo</t>
         </is>
       </c>
-      <c r="B22" s="21" t="inlineStr">
-        <is>
-          <t>Volumen Personal mínimo que TÚ debes producir directamente cada mes (pendiente: convertir a puntos en próxima iteración).</t>
+      <c r="B22" s="24" t="inlineStr">
+        <is>
+          <t>Volumen Personal mínimo que TÚ debes producir directamente cada mes (pendiente convertir a puntos).</t>
         </is>
       </c>
     </row>
     <row r="23" ht="22" customHeight="1">
-      <c r="A23" s="20" t="inlineStr">
+      <c r="A23" s="23" t="inlineStr">
         <is>
           <t>Patrocinados activos</t>
         </is>
       </c>
-      <c r="B23" s="21" t="inlineStr">
+      <c r="B23" s="24" t="inlineStr">
         <is>
           <t>Socios que TÚ trajiste personalmente y que cumplen su PV mínimo ese mes.</t>
         </is>
       </c>
     </row>
     <row r="24" ht="22" customHeight="1">
-      <c r="A24" s="20" t="inlineStr">
+      <c r="A24" s="23" t="inlineStr">
         <is>
           <t>Piernas calificadas</t>
         </is>
       </c>
-      <c r="B24" s="21" t="inlineStr">
+      <c r="B24" s="24" t="inlineStr">
         <is>
           <t>Ramas independientes (downlines de patrocinados directos distintos) donde alguien dentro alcanza el rango indicado entre paréntesis.</t>
         </is>
       </c>
     </row>
     <row r="25" ht="22" customHeight="1">
-      <c r="A25" s="20" t="inlineStr">
-        <is>
-          <t>Cobro estimado</t>
-        </is>
-      </c>
-      <c r="B25" s="21" t="inlineStr">
-        <is>
-          <t>Ingreso aproximado mensual proyectado por la combinación FSB + Uninivel + Pool.</t>
+      <c r="A25" s="23" t="inlineStr">
+        <is>
+          <t>Bono Gift (editable)</t>
+        </is>
+      </c>
+      <c r="B25" s="24" t="inlineStr">
+        <is>
+          <t>Bono adicional discrecional. Edita el valor en USD (celda azul) y el Cobro estimado se recalcula automáticamente sumando el bono al min y al max.</t>
         </is>
       </c>
     </row>
     <row r="26" ht="22" customHeight="1">
-      <c r="A26" s="20" t="inlineStr">
+      <c r="A26" s="23" t="inlineStr">
+        <is>
+          <t>Cobro estimado (fórmula)</t>
+        </is>
+      </c>
+      <c r="B26" s="24" t="inlineStr">
+        <is>
+          <t>Min = 22% × PV/mes del rango actual + Bono Gift. Max = 22% × PV/mes del siguiente rango + Bono Gift. Leyenda solo muestra el mínimo con '+' (sin tope).</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="22" customHeight="1">
+      <c r="A27" s="23" t="inlineStr">
         <is>
           <t>Regla 50/50 (sugerida)</t>
         </is>
       </c>
-      <c r="B26" s="21" t="inlineStr">
+      <c r="B27" s="24" t="inlineStr">
         <is>
           <t>Ninguna pierna puede aportar más del 50% del volumen requerido para el rango.</t>
         </is>
       </c>
     </row>
-    <row r="28">
-      <c r="A28" s="19" t="inlineStr">
+    <row r="29">
+      <c r="A29" s="22" t="inlineStr">
         <is>
           <t>PENDIENTES DE CONFIRMAR</t>
         </is>
       </c>
     </row>
-    <row r="29" ht="20" customHeight="1">
-      <c r="A29" s="22" t="inlineStr">
+    <row r="30" ht="20" customHeight="1">
+      <c r="A30" s="25" t="inlineStr">
         <is>
           <t>☐  PV mínimos por rango (¿OK los valores propuestos?)</t>
         </is>
       </c>
     </row>
-    <row r="30" ht="20" customHeight="1">
-      <c r="A30" s="22" t="inlineStr">
+    <row r="31" ht="20" customHeight="1">
+      <c r="A31" s="25" t="inlineStr">
         <is>
           <t>☐  Número de patrocinados activos por rango</t>
         </is>
       </c>
     </row>
-    <row r="31" ht="20" customHeight="1">
-      <c r="A31" s="22" t="inlineStr">
+    <row r="32" ht="20" customHeight="1">
+      <c r="A32" s="25" t="inlineStr">
         <is>
           <t>☐  Piernas calificadas y su rango exigido</t>
         </is>
       </c>
     </row>
-    <row r="32" ht="20" customHeight="1">
-      <c r="A32" s="22" t="inlineStr">
+    <row r="33" ht="20" customHeight="1">
+      <c r="A33" s="25" t="inlineStr">
         <is>
           <t>☐  Activar/no activar regla 50/50</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="13">
-    <mergeCell ref="B24:G24"/>
-    <mergeCell ref="A32:G32"/>
-    <mergeCell ref="B20:G20"/>
-    <mergeCell ref="A1:G1"/>
-    <mergeCell ref="B22:G22"/>
-    <mergeCell ref="A31:G31"/>
-    <mergeCell ref="B23:G23"/>
-    <mergeCell ref="A30:G30"/>
-    <mergeCell ref="A2:G2"/>
-    <mergeCell ref="B26:G26"/>
-    <mergeCell ref="A29:G29"/>
-    <mergeCell ref="B21:G21"/>
-    <mergeCell ref="B25:G25"/>
+  <mergeCells count="14">
+    <mergeCell ref="B22:H22"/>
+    <mergeCell ref="A30:H30"/>
+    <mergeCell ref="B26:H26"/>
+    <mergeCell ref="B27:H27"/>
+    <mergeCell ref="B21:H21"/>
+    <mergeCell ref="A2:H2"/>
+    <mergeCell ref="A31:H31"/>
+    <mergeCell ref="B24:H24"/>
+    <mergeCell ref="A33:H33"/>
+    <mergeCell ref="B25:H25"/>
+    <mergeCell ref="A1:H1"/>
+    <mergeCell ref="A32:H32"/>
+    <mergeCell ref="B20:H20"/>
+    <mergeCell ref="B23:H23"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter>

</xml_diff>